<commit_message>
resolve example error 389ebd4792fb95d9bf9b663d84e2943b628feec6
</commit_message>
<xml_diff>
--- a/ig/nr-resolve-example-error/StructureDefinition-mesures-observation-steps-by-day.xlsx
+++ b/ig/nr-resolve-example-error/StructureDefinition-mesures-observation-steps-by-day.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-01T17:10:19+00:00</t>
+    <t>2024-02-02T09:57:39+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1131,8 +1131,8 @@
     <t>Observation.code.coding</t>
   </si>
   <si>
-    <t>value:code}
-value:system}</t>
+    <t>pattern:code}
+pattern:system}</t>
   </si>
   <si>
     <t>Observation.code.coding:stepsBDCode</t>

</xml_diff>